<commit_message>
Finalising functions in stage 6 :)
</commit_message>
<xml_diff>
--- a/TOR330 Data/5. Clean Data for Data Visualisation/Anomalies Tracker/TOR330_finisher_anomalies.xlsx
+++ b/TOR330 Data/5. Clean Data for Data Visualisation/Anomalies Tracker/TOR330_finisher_anomalies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="88">
   <si>
     <t>Name</t>
   </si>
@@ -212,6 +212,30 @@
   </si>
   <si>
     <t>Smith Jonathan</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>275</t>
+  </si>
+  <si>
+    <t>493</t>
+  </si>
+  <si>
+    <t>540</t>
+  </si>
+  <si>
+    <t>665</t>
+  </si>
+  <si>
+    <t>1105</t>
+  </si>
+  <si>
+    <t>1143</t>
+  </si>
+  <si>
+    <t>1321</t>
   </si>
   <si>
     <t>F</t>
@@ -615,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BF9"/>
+  <dimension ref="A1:BF41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:58">
@@ -802,19 +826,19 @@
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" t="s">
-        <v>75</v>
+        <v>76</v>
+      </c>
+      <c r="E2">
+        <v>2023</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G2" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -882,19 +906,19 @@
         <v>275</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" t="s">
-        <v>75</v>
+        <v>77</v>
+      </c>
+      <c r="E3">
+        <v>2023</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -989,19 +1013,19 @@
         <v>493</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E4" t="s">
-        <v>75</v>
+        <v>78</v>
+      </c>
+      <c r="E4">
+        <v>2023</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1087,19 +1111,19 @@
         <v>540</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" t="s">
-        <v>75</v>
+        <v>77</v>
+      </c>
+      <c r="E5">
+        <v>2023</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1137,19 +1161,19 @@
         <v>665</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E6" t="s">
-        <v>75</v>
+        <v>79</v>
+      </c>
+      <c r="E6">
+        <v>2023</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H6" t="b">
         <v>1</v>
@@ -1214,19 +1238,19 @@
         <v>1105</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7" t="s">
-        <v>75</v>
+        <v>80</v>
+      </c>
+      <c r="E7">
+        <v>2023</v>
       </c>
       <c r="F7" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H7" t="b">
         <v>1</v>
@@ -1273,19 +1297,19 @@
         <v>1143</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" t="s">
-        <v>75</v>
+        <v>81</v>
+      </c>
+      <c r="E8">
+        <v>2023</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G8" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
@@ -1371,19 +1395,19 @@
         <v>1321</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" t="s">
-        <v>75</v>
+        <v>82</v>
+      </c>
+      <c r="E9">
+        <v>2023</v>
       </c>
       <c r="F9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G9" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -1440,6 +1464,2602 @@
         <v>45181.72148148148</v>
       </c>
       <c r="BF9" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="10" spans="1:58">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10">
+        <v>2023</v>
+      </c>
+      <c r="F10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J10" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K10" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L10" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M10" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N10" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O10" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P10" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R10" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S10" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T10" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U10" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V10" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W10" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X10" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z10" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF10" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="11" spans="1:58">
+      <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11">
+        <v>275</v>
+      </c>
+      <c r="C11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11">
+        <v>2023</v>
+      </c>
+      <c r="F11" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J11" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K11" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L11" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M11" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N11" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O11" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P11" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R11" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S11" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T11" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U11" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V11" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W11" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X11" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y11" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z11" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA11" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB11" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC11" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD11" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE11" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF11" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG11" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK11" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF11" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="12" spans="1:58">
+      <c r="A12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12">
+        <v>493</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12">
+        <v>2023</v>
+      </c>
+      <c r="F12" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J12" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K12" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L12" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M12" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N12" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O12" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P12" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R12" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S12" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T12" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U12" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V12" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W12" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X12" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y12" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z12" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA12" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB12" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC12" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD12" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE12" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF12" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="13" spans="1:58">
+      <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13">
+        <v>540</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13">
+        <v>2023</v>
+      </c>
+      <c r="F13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J13" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K13" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L13" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M13" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N13" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O13" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF13" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="14" spans="1:58">
+      <c r="A14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14">
+        <v>665</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14">
+        <v>2023</v>
+      </c>
+      <c r="F14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" t="s">
+        <v>86</v>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J14" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K14" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L14" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M14" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N14" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O14" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P14" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R14" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S14" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T14" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V14" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W14" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X14" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z14" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF14" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="15" spans="1:58">
+      <c r="A15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15">
+        <v>1105</v>
+      </c>
+      <c r="C15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15">
+        <v>2023</v>
+      </c>
+      <c r="F15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J15" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K15" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L15" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M15" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N15" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O15" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R15" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S15" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF15" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="16" spans="1:58">
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16">
+        <v>1143</v>
+      </c>
+      <c r="C16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16">
+        <v>2023</v>
+      </c>
+      <c r="F16" t="s">
+        <v>84</v>
+      </c>
+      <c r="G16" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J16" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K16" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L16" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M16" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N16" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O16" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R16" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S16" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T16" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U16" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V16" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W16" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X16" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y16" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z16" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA16" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB16" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD16" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE16" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF16" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG16" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF16" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="17" spans="1:58">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17">
+        <v>1321</v>
+      </c>
+      <c r="C17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E17">
+        <v>2023</v>
+      </c>
+      <c r="F17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17" t="s">
+        <v>87</v>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J17" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K17" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L17" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M17" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N17" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O17" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P17" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R17" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S17" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T17" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U17" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V17" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W17" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X17" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA17" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF17" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="18" spans="1:58">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18">
+        <v>48</v>
+      </c>
+      <c r="C18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18">
+        <v>2023</v>
+      </c>
+      <c r="F18" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J18" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K18" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L18" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M18" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N18" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O18" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P18" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R18" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S18" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T18" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U18" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V18" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W18" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X18" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z18" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF18" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="19" spans="1:58">
+      <c r="A19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19">
+        <v>275</v>
+      </c>
+      <c r="C19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19">
+        <v>2023</v>
+      </c>
+      <c r="F19" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" t="s">
+        <v>85</v>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J19" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K19" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L19" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M19" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N19" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O19" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P19" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R19" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S19" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T19" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U19" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V19" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W19" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X19" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y19" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA19" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC19" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD19" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE19" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF19" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG19" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK19" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF19" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="20" spans="1:58">
+      <c r="A20" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20">
+        <v>493</v>
+      </c>
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20">
+        <v>2023</v>
+      </c>
+      <c r="F20" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" t="s">
+        <v>85</v>
+      </c>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J20" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K20" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L20" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M20" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N20" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O20" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P20" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R20" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S20" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T20" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U20" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V20" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W20" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X20" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y20" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z20" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA20" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB20" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC20" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD20" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE20" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF20" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="21" spans="1:58">
+      <c r="A21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21">
+        <v>540</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21">
+        <v>2023</v>
+      </c>
+      <c r="F21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G21" t="s">
+        <v>86</v>
+      </c>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J21" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K21" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L21" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M21" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N21" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O21" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF21" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="22" spans="1:58">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22">
+        <v>665</v>
+      </c>
+      <c r="C22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22">
+        <v>2023</v>
+      </c>
+      <c r="F22" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" t="s">
+        <v>86</v>
+      </c>
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J22" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K22" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L22" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M22" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N22" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O22" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P22" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R22" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S22" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T22" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V22" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W22" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X22" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z22" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF22" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="23" spans="1:58">
+      <c r="A23" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23">
+        <v>1105</v>
+      </c>
+      <c r="C23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23">
+        <v>2023</v>
+      </c>
+      <c r="F23" t="s">
+        <v>84</v>
+      </c>
+      <c r="G23" t="s">
+        <v>86</v>
+      </c>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J23" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K23" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L23" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M23" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N23" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O23" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R23" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S23" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF23" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="24" spans="1:58">
+      <c r="A24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24">
+        <v>1143</v>
+      </c>
+      <c r="C24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" t="s">
+        <v>81</v>
+      </c>
+      <c r="E24">
+        <v>2023</v>
+      </c>
+      <c r="F24" t="s">
+        <v>84</v>
+      </c>
+      <c r="G24" t="s">
+        <v>87</v>
+      </c>
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J24" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K24" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L24" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M24" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N24" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O24" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R24" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S24" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T24" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U24" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V24" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W24" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X24" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y24" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z24" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA24" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB24" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD24" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE24" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF24" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG24" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF24" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="25" spans="1:58">
+      <c r="A25" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25">
+        <v>1321</v>
+      </c>
+      <c r="C25" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25">
+        <v>2023</v>
+      </c>
+      <c r="F25" t="s">
+        <v>84</v>
+      </c>
+      <c r="G25" t="s">
+        <v>87</v>
+      </c>
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J25" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K25" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L25" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M25" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N25" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O25" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P25" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R25" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S25" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T25" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U25" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V25" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W25" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X25" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA25" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF25" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="26" spans="1:58">
+      <c r="A26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26">
+        <v>48</v>
+      </c>
+      <c r="C26" t="s">
+        <v>74</v>
+      </c>
+      <c r="D26" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26">
+        <v>2023</v>
+      </c>
+      <c r="F26" t="s">
+        <v>84</v>
+      </c>
+      <c r="G26" t="s">
+        <v>85</v>
+      </c>
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J26" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K26" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L26" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M26" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N26" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O26" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P26" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R26" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S26" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T26" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U26" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V26" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W26" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X26" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z26" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF26" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="27" spans="1:58">
+      <c r="A27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27">
+        <v>275</v>
+      </c>
+      <c r="C27" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27">
+        <v>2023</v>
+      </c>
+      <c r="F27" t="s">
+        <v>84</v>
+      </c>
+      <c r="G27" t="s">
+        <v>85</v>
+      </c>
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J27" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K27" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L27" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M27" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N27" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O27" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P27" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R27" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S27" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T27" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U27" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V27" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W27" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X27" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y27" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z27" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA27" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB27" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC27" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD27" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE27" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF27" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG27" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK27" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF27" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="28" spans="1:58">
+      <c r="A28" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28">
+        <v>493</v>
+      </c>
+      <c r="C28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28">
+        <v>2023</v>
+      </c>
+      <c r="F28" t="s">
+        <v>84</v>
+      </c>
+      <c r="G28" t="s">
+        <v>85</v>
+      </c>
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J28" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K28" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L28" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M28" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N28" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O28" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P28" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R28" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S28" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T28" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U28" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V28" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W28" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X28" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y28" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z28" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA28" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB28" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC28" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD28" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE28" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF28" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="29" spans="1:58">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29">
+        <v>540</v>
+      </c>
+      <c r="C29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E29">
+        <v>2023</v>
+      </c>
+      <c r="F29" t="s">
+        <v>84</v>
+      </c>
+      <c r="G29" t="s">
+        <v>86</v>
+      </c>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J29" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K29" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L29" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M29" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N29" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O29" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF29" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="30" spans="1:58">
+      <c r="A30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30">
+        <v>665</v>
+      </c>
+      <c r="C30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E30">
+        <v>2023</v>
+      </c>
+      <c r="F30" t="s">
+        <v>84</v>
+      </c>
+      <c r="G30" t="s">
+        <v>86</v>
+      </c>
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J30" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K30" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L30" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M30" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N30" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O30" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P30" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R30" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S30" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T30" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V30" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W30" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X30" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z30" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF30" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="31" spans="1:58">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31">
+        <v>1105</v>
+      </c>
+      <c r="C31" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" t="s">
+        <v>80</v>
+      </c>
+      <c r="E31">
+        <v>2023</v>
+      </c>
+      <c r="F31" t="s">
+        <v>84</v>
+      </c>
+      <c r="G31" t="s">
+        <v>86</v>
+      </c>
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J31" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K31" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L31" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M31" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N31" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O31" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R31" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S31" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF31" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="32" spans="1:58">
+      <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32">
+        <v>1143</v>
+      </c>
+      <c r="C32" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" t="s">
+        <v>81</v>
+      </c>
+      <c r="E32">
+        <v>2023</v>
+      </c>
+      <c r="F32" t="s">
+        <v>84</v>
+      </c>
+      <c r="G32" t="s">
+        <v>87</v>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J32" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K32" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L32" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M32" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N32" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O32" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R32" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S32" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T32" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U32" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V32" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W32" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X32" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y32" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z32" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA32" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB32" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD32" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE32" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF32" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG32" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF32" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="33" spans="1:58">
+      <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33">
+        <v>1321</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" t="s">
+        <v>82</v>
+      </c>
+      <c r="E33">
+        <v>2023</v>
+      </c>
+      <c r="F33" t="s">
+        <v>84</v>
+      </c>
+      <c r="G33" t="s">
+        <v>87</v>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J33" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K33" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L33" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M33" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N33" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O33" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P33" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R33" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S33" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T33" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U33" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V33" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W33" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X33" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA33" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF33" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="34" spans="1:58">
+      <c r="A34" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" t="s">
+        <v>76</v>
+      </c>
+      <c r="E34" t="s">
+        <v>83</v>
+      </c>
+      <c r="F34" t="s">
+        <v>84</v>
+      </c>
+      <c r="G34" t="s">
+        <v>85</v>
+      </c>
+      <c r="H34" t="b">
+        <v>1</v>
+      </c>
+      <c r="I34" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J34" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K34" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L34" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M34" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N34" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O34" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P34" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R34" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S34" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T34" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U34" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V34" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W34" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X34" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z34" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF34" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="35" spans="1:58">
+      <c r="A35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" t="s">
+        <v>77</v>
+      </c>
+      <c r="E35" t="s">
+        <v>83</v>
+      </c>
+      <c r="F35" t="s">
+        <v>84</v>
+      </c>
+      <c r="G35" t="s">
+        <v>85</v>
+      </c>
+      <c r="H35" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J35" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K35" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L35" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M35" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N35" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O35" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P35" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R35" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S35" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T35" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U35" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V35" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W35" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X35" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y35" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z35" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA35" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB35" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC35" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD35" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE35" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF35" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG35" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK35" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF35" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="36" spans="1:58">
+      <c r="A36" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E36" t="s">
+        <v>83</v>
+      </c>
+      <c r="F36" t="s">
+        <v>84</v>
+      </c>
+      <c r="G36" t="s">
+        <v>85</v>
+      </c>
+      <c r="H36" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J36" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K36" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L36" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M36" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N36" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O36" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P36" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R36" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S36" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T36" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U36" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V36" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W36" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X36" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y36" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z36" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA36" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB36" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC36" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD36" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE36" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF36" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="37" spans="1:58">
+      <c r="A37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" t="s">
+        <v>69</v>
+      </c>
+      <c r="C37" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" t="s">
+        <v>77</v>
+      </c>
+      <c r="E37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F37" t="s">
+        <v>84</v>
+      </c>
+      <c r="G37" t="s">
+        <v>86</v>
+      </c>
+      <c r="H37" t="b">
+        <v>1</v>
+      </c>
+      <c r="I37" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J37" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K37" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L37" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M37" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N37" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O37" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF37" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="38" spans="1:58">
+      <c r="A38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" t="s">
+        <v>74</v>
+      </c>
+      <c r="D38" t="s">
+        <v>79</v>
+      </c>
+      <c r="E38" t="s">
+        <v>83</v>
+      </c>
+      <c r="F38" t="s">
+        <v>84</v>
+      </c>
+      <c r="G38" t="s">
+        <v>86</v>
+      </c>
+      <c r="H38" t="b">
+        <v>1</v>
+      </c>
+      <c r="I38" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J38" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K38" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L38" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M38" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N38" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O38" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P38" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R38" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S38" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T38" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V38" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W38" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X38" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z38" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF38" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="39" spans="1:58">
+      <c r="A39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" t="s">
+        <v>74</v>
+      </c>
+      <c r="D39" t="s">
+        <v>80</v>
+      </c>
+      <c r="E39" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39" t="s">
+        <v>84</v>
+      </c>
+      <c r="G39" t="s">
+        <v>86</v>
+      </c>
+      <c r="H39" t="b">
+        <v>1</v>
+      </c>
+      <c r="I39" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J39" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K39" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L39" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M39" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N39" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O39" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R39" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S39" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF39" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="40" spans="1:58">
+      <c r="A40" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" t="s">
+        <v>81</v>
+      </c>
+      <c r="E40" t="s">
+        <v>83</v>
+      </c>
+      <c r="F40" t="s">
+        <v>84</v>
+      </c>
+      <c r="G40" t="s">
+        <v>87</v>
+      </c>
+      <c r="H40" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J40" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K40" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L40" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M40" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N40" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O40" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R40" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S40" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T40" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U40" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V40" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W40" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X40" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y40" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z40" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA40" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB40" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD40" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE40" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF40" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG40" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF40" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="41" spans="1:58">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" t="s">
+        <v>82</v>
+      </c>
+      <c r="E41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F41" t="s">
+        <v>84</v>
+      </c>
+      <c r="G41" t="s">
+        <v>87</v>
+      </c>
+      <c r="H41" t="b">
+        <v>1</v>
+      </c>
+      <c r="I41" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J41" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K41" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L41" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M41" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N41" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O41" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P41" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R41" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S41" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T41" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U41" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V41" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W41" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X41" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA41" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF41" s="2">
         <v>45184.58322916667</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding databases back into github
</commit_message>
<xml_diff>
--- a/TOR330 Data/5. Clean Data for Data Visualisation/Anomalies Tracker/TOR330_finisher_anomalies.xlsx
+++ b/TOR330 Data/5. Clean Data for Data Visualisation/Anomalies Tracker/TOR330_finisher_anomalies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="92">
   <si>
     <t>Name</t>
   </si>
@@ -223,10 +223,22 @@
     <t>Cagna Andrea</t>
   </si>
   <si>
-    <t>99</t>
-  </si>
-  <si>
-    <t>1547</t>
+    <t>Pier Franco Franciscono</t>
+  </si>
+  <si>
+    <t>Satoko Uchida</t>
+  </si>
+  <si>
+    <t>Franciscono Pier Franco</t>
+  </si>
+  <si>
+    <t>Uchida Satoko</t>
+  </si>
+  <si>
+    <t>1306</t>
+  </si>
+  <si>
+    <t>1360</t>
   </si>
   <si>
     <t>M</t>
@@ -262,7 +274,7 @@
     <t>IT</t>
   </si>
   <si>
-    <t>2024</t>
+    <t>2025</t>
   </si>
   <si>
     <t>TOR330</t>
@@ -639,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BF13"/>
+  <dimension ref="A1:BF49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:58">
@@ -826,19 +838,19 @@
         <v>668</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E2">
         <v>2021</v>
       </c>
       <c r="F2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -930,19 +942,19 @@
         <v>668</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -1034,19 +1046,19 @@
         <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E4">
         <v>2023</v>
       </c>
       <c r="F4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1114,19 +1126,19 @@
         <v>275</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E5">
         <v>2023</v>
       </c>
       <c r="F5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1221,19 +1233,19 @@
         <v>493</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E6">
         <v>2023</v>
       </c>
       <c r="F6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H6" t="b">
         <v>1</v>
@@ -1319,19 +1331,19 @@
         <v>540</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E7">
         <v>2023</v>
       </c>
       <c r="F7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H7" t="b">
         <v>1</v>
@@ -1369,19 +1381,19 @@
         <v>665</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E8">
         <v>2023</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
@@ -1446,19 +1458,19 @@
         <v>1105</v>
       </c>
       <c r="C9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E9">
         <v>2023</v>
       </c>
       <c r="F9" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -1505,19 +1517,19 @@
         <v>1143</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E10">
         <v>2023</v>
       </c>
       <c r="F10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G10" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H10" t="b">
         <v>1</v>
@@ -1603,19 +1615,19 @@
         <v>1321</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E11">
         <v>2023</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G11" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
@@ -1679,23 +1691,23 @@
       <c r="A12" t="s">
         <v>67</v>
       </c>
-      <c r="B12" t="s">
-        <v>69</v>
+      <c r="B12">
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
-      </c>
-      <c r="E12" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="E12">
+        <v>2024</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G12" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H12" t="b">
         <v>1</v>
@@ -1795,23 +1807,23 @@
       <c r="A13" t="s">
         <v>68</v>
       </c>
-      <c r="B13" t="s">
-        <v>70</v>
+      <c r="B13">
+        <v>1547</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" t="s">
-        <v>82</v>
+        <v>85</v>
+      </c>
+      <c r="E13">
+        <v>2024</v>
       </c>
       <c r="F13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G13" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
@@ -1857,6 +1869,3213 @@
       </c>
       <c r="BF13" s="2">
         <v>45548.75009259259</v>
+      </c>
+    </row>
+    <row r="14" spans="1:58">
+      <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14">
+        <v>1306</v>
+      </c>
+      <c r="C14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14">
+        <v>2025</v>
+      </c>
+      <c r="F14" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2">
+        <v>45914.47542606481</v>
+      </c>
+      <c r="J14" s="2">
+        <v>45914.62513768519</v>
+      </c>
+      <c r="K14" s="2">
+        <v>45914.66811888889</v>
+      </c>
+      <c r="L14" s="2">
+        <v>45914.7943594676</v>
+      </c>
+      <c r="M14" s="2">
+        <v>45915.11259197917</v>
+      </c>
+      <c r="N14" s="2">
+        <v>45915.18046519676</v>
+      </c>
+      <c r="O14" s="2">
+        <v>45915.23756817129</v>
+      </c>
+      <c r="P14" s="2">
+        <v>45915.33654960648</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>45915.46181254629</v>
+      </c>
+      <c r="R14" s="2">
+        <v>45915.75465270833</v>
+      </c>
+      <c r="T14" s="2">
+        <v>45916.23184403935</v>
+      </c>
+      <c r="U14" s="2">
+        <v>45916.2964321875</v>
+      </c>
+      <c r="V14" s="2">
+        <v>45916.3633465625</v>
+      </c>
+      <c r="W14" s="2">
+        <v>45916.59064263889</v>
+      </c>
+      <c r="X14" s="2">
+        <v>45916.67155491898</v>
+      </c>
+      <c r="Y14" s="2">
+        <v>45916.76256023148</v>
+      </c>
+      <c r="Z14" s="2">
+        <v>45916.87893012731</v>
+      </c>
+      <c r="AA14" s="2">
+        <v>45917.01325516203</v>
+      </c>
+      <c r="AB14" s="2">
+        <v>45917.09894671296</v>
+      </c>
+      <c r="AC14" s="2">
+        <v>45917.2452054051</v>
+      </c>
+      <c r="AD14" s="2">
+        <v>45917.37764478009</v>
+      </c>
+      <c r="AE14" s="2">
+        <v>45917.56345918981</v>
+      </c>
+      <c r="AG14" s="2">
+        <v>45917.86822302084</v>
+      </c>
+      <c r="AU14" s="2">
+        <v>45914.91300321759</v>
+      </c>
+      <c r="BF14" s="2">
+        <v>45920.66509259259</v>
+      </c>
+    </row>
+    <row r="15" spans="1:58">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15">
+        <v>1360</v>
+      </c>
+      <c r="C15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" t="s">
+        <v>82</v>
+      </c>
+      <c r="E15">
+        <v>2025</v>
+      </c>
+      <c r="F15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>89</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
+        <v>45914.48986140046</v>
+      </c>
+      <c r="J15" s="2">
+        <v>45914.63592015046</v>
+      </c>
+      <c r="K15" s="2">
+        <v>45914.67685524306</v>
+      </c>
+      <c r="L15" s="2">
+        <v>45914.78852579861</v>
+      </c>
+      <c r="M15" s="2">
+        <v>45915.08358268518</v>
+      </c>
+      <c r="N15" s="2">
+        <v>45915.08100641204</v>
+      </c>
+      <c r="O15" s="2">
+        <v>45915.18725445602</v>
+      </c>
+      <c r="P15" s="2">
+        <v>45915.26926759259</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>45915.37480168982</v>
+      </c>
+      <c r="R15" s="2">
+        <v>45915.60506037037</v>
+      </c>
+      <c r="T15" s="2">
+        <v>45915.97002079861</v>
+      </c>
+      <c r="V15" s="2">
+        <v>45916.20189703703</v>
+      </c>
+      <c r="W15" s="2">
+        <v>45916.39650483796</v>
+      </c>
+      <c r="X15" s="2">
+        <v>45916.45933371528</v>
+      </c>
+      <c r="Y15" s="2">
+        <v>45916.53816135417</v>
+      </c>
+      <c r="Z15" s="2">
+        <v>45916.64014879629</v>
+      </c>
+      <c r="AA15" s="2">
+        <v>45916.78958375</v>
+      </c>
+      <c r="AB15" s="2">
+        <v>45916.8618480787</v>
+      </c>
+      <c r="AC15" s="2">
+        <v>45916.96367357639</v>
+      </c>
+      <c r="AD15" s="2">
+        <v>45917.06572414352</v>
+      </c>
+      <c r="AE15" s="2">
+        <v>45917.23132472222</v>
+      </c>
+      <c r="AF15" s="2">
+        <v>45917.41728608796</v>
+      </c>
+      <c r="AG15" s="2">
+        <v>45917.5006153125</v>
+      </c>
+      <c r="AH15" s="2">
+        <v>45917.59454695602</v>
+      </c>
+      <c r="AI15" s="2">
+        <v>45917.71892535879</v>
+      </c>
+      <c r="AJ15" s="2">
+        <v>45917.82246778935</v>
+      </c>
+      <c r="AK15" s="2">
+        <v>45917.97690543981</v>
+      </c>
+      <c r="AL15" s="2">
+        <v>45918.10435318287</v>
+      </c>
+      <c r="AU15" s="2">
+        <v>45914.87498131944</v>
+      </c>
+      <c r="BF15" s="2">
+        <v>45920.46710648148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:58">
+      <c r="A16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16">
+        <v>1306</v>
+      </c>
+      <c r="C16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16">
+        <v>2025</v>
+      </c>
+      <c r="F16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" t="s">
+        <v>88</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2">
+        <v>45914.47542606481</v>
+      </c>
+      <c r="J16" s="2">
+        <v>45914.62513768519</v>
+      </c>
+      <c r="K16" s="2">
+        <v>45914.66811888889</v>
+      </c>
+      <c r="L16" s="2">
+        <v>45914.7943594676</v>
+      </c>
+      <c r="M16" s="2">
+        <v>45915.11259197917</v>
+      </c>
+      <c r="N16" s="2">
+        <v>45915.18046519676</v>
+      </c>
+      <c r="O16" s="2">
+        <v>45915.23756817129</v>
+      </c>
+      <c r="P16" s="2">
+        <v>45915.33654960648</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>45915.46181254629</v>
+      </c>
+      <c r="R16" s="2">
+        <v>45915.75465270833</v>
+      </c>
+      <c r="T16" s="2">
+        <v>45916.23184403935</v>
+      </c>
+      <c r="U16" s="2">
+        <v>45916.2964321875</v>
+      </c>
+      <c r="V16" s="2">
+        <v>45916.3633465625</v>
+      </c>
+      <c r="W16" s="2">
+        <v>45916.59064263889</v>
+      </c>
+      <c r="X16" s="2">
+        <v>45916.67155491898</v>
+      </c>
+      <c r="Y16" s="2">
+        <v>45916.76256023148</v>
+      </c>
+      <c r="Z16" s="2">
+        <v>45916.87893012731</v>
+      </c>
+      <c r="AA16" s="2">
+        <v>45917.01325516203</v>
+      </c>
+      <c r="AB16" s="2">
+        <v>45917.09894671296</v>
+      </c>
+      <c r="AC16" s="2">
+        <v>45917.2452054051</v>
+      </c>
+      <c r="AD16" s="2">
+        <v>45917.37764478009</v>
+      </c>
+      <c r="AE16" s="2">
+        <v>45917.56345918981</v>
+      </c>
+      <c r="AG16" s="2">
+        <v>45917.86822302084</v>
+      </c>
+      <c r="AU16" s="2">
+        <v>45914.91300321759</v>
+      </c>
+      <c r="BF16" s="2">
+        <v>45920.66509259259</v>
+      </c>
+    </row>
+    <row r="17" spans="1:58">
+      <c r="A17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17">
+        <v>1360</v>
+      </c>
+      <c r="C17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E17">
+        <v>2025</v>
+      </c>
+      <c r="F17" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" t="s">
+        <v>89</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2">
+        <v>45914.48986140046</v>
+      </c>
+      <c r="J17" s="2">
+        <v>45914.63592015046</v>
+      </c>
+      <c r="K17" s="2">
+        <v>45914.67685524306</v>
+      </c>
+      <c r="L17" s="2">
+        <v>45914.78852579861</v>
+      </c>
+      <c r="M17" s="2">
+        <v>45915.08358268518</v>
+      </c>
+      <c r="N17" s="2">
+        <v>45915.08100641204</v>
+      </c>
+      <c r="O17" s="2">
+        <v>45915.18725445602</v>
+      </c>
+      <c r="P17" s="2">
+        <v>45915.26926759259</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>45915.37480168982</v>
+      </c>
+      <c r="R17" s="2">
+        <v>45915.60506037037</v>
+      </c>
+      <c r="T17" s="2">
+        <v>45915.97002079861</v>
+      </c>
+      <c r="V17" s="2">
+        <v>45916.20189703703</v>
+      </c>
+      <c r="W17" s="2">
+        <v>45916.39650483796</v>
+      </c>
+      <c r="X17" s="2">
+        <v>45916.45933371528</v>
+      </c>
+      <c r="Y17" s="2">
+        <v>45916.53816135417</v>
+      </c>
+      <c r="Z17" s="2">
+        <v>45916.64014879629</v>
+      </c>
+      <c r="AA17" s="2">
+        <v>45916.78958375</v>
+      </c>
+      <c r="AB17" s="2">
+        <v>45916.8618480787</v>
+      </c>
+      <c r="AC17" s="2">
+        <v>45916.96367357639</v>
+      </c>
+      <c r="AD17" s="2">
+        <v>45917.06572414352</v>
+      </c>
+      <c r="AE17" s="2">
+        <v>45917.23132472222</v>
+      </c>
+      <c r="AF17" s="2">
+        <v>45917.41728608796</v>
+      </c>
+      <c r="AG17" s="2">
+        <v>45917.5006153125</v>
+      </c>
+      <c r="AH17" s="2">
+        <v>45917.59454695602</v>
+      </c>
+      <c r="AI17" s="2">
+        <v>45917.71892535879</v>
+      </c>
+      <c r="AJ17" s="2">
+        <v>45917.82246778935</v>
+      </c>
+      <c r="AK17" s="2">
+        <v>45917.97690543981</v>
+      </c>
+      <c r="AL17" s="2">
+        <v>45918.10435318287</v>
+      </c>
+      <c r="AU17" s="2">
+        <v>45914.87498131944</v>
+      </c>
+      <c r="BF17" s="2">
+        <v>45920.46710648148</v>
+      </c>
+    </row>
+    <row r="18" spans="1:58">
+      <c r="A18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18">
+        <v>1306</v>
+      </c>
+      <c r="C18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" t="s">
+        <v>85</v>
+      </c>
+      <c r="E18">
+        <v>2025</v>
+      </c>
+      <c r="F18" t="s">
+        <v>87</v>
+      </c>
+      <c r="G18" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2">
+        <v>45914.47542606481</v>
+      </c>
+      <c r="J18" s="2">
+        <v>45914.62513768519</v>
+      </c>
+      <c r="K18" s="2">
+        <v>45914.66811888889</v>
+      </c>
+      <c r="L18" s="2">
+        <v>45914.7943594676</v>
+      </c>
+      <c r="M18" s="2">
+        <v>45915.11259197917</v>
+      </c>
+      <c r="N18" s="2">
+        <v>45915.18046519676</v>
+      </c>
+      <c r="O18" s="2">
+        <v>45915.23756817129</v>
+      </c>
+      <c r="P18" s="2">
+        <v>45915.33654960648</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>45915.46181254629</v>
+      </c>
+      <c r="R18" s="2">
+        <v>45915.75465270833</v>
+      </c>
+      <c r="T18" s="2">
+        <v>45916.23184403935</v>
+      </c>
+      <c r="U18" s="2">
+        <v>45916.2964321875</v>
+      </c>
+      <c r="V18" s="2">
+        <v>45916.3633465625</v>
+      </c>
+      <c r="W18" s="2">
+        <v>45916.59064263889</v>
+      </c>
+      <c r="X18" s="2">
+        <v>45916.67155491898</v>
+      </c>
+      <c r="Y18" s="2">
+        <v>45916.76256023148</v>
+      </c>
+      <c r="Z18" s="2">
+        <v>45916.87893012731</v>
+      </c>
+      <c r="AA18" s="2">
+        <v>45917.01325516203</v>
+      </c>
+      <c r="AB18" s="2">
+        <v>45917.09894671296</v>
+      </c>
+      <c r="AC18" s="2">
+        <v>45917.2452054051</v>
+      </c>
+      <c r="AD18" s="2">
+        <v>45917.37764478009</v>
+      </c>
+      <c r="AE18" s="2">
+        <v>45917.56345918981</v>
+      </c>
+      <c r="AG18" s="2">
+        <v>45917.86822302084</v>
+      </c>
+      <c r="AU18" s="2">
+        <v>45914.91300321759</v>
+      </c>
+      <c r="BF18" s="2">
+        <v>45920.66509259259</v>
+      </c>
+    </row>
+    <row r="19" spans="1:58">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19">
+        <v>1360</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19">
+        <v>2025</v>
+      </c>
+      <c r="F19" t="s">
+        <v>87</v>
+      </c>
+      <c r="G19" t="s">
+        <v>89</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2">
+        <v>45914.48986140046</v>
+      </c>
+      <c r="J19" s="2">
+        <v>45914.63592015046</v>
+      </c>
+      <c r="K19" s="2">
+        <v>45914.67685524306</v>
+      </c>
+      <c r="L19" s="2">
+        <v>45914.78852579861</v>
+      </c>
+      <c r="M19" s="2">
+        <v>45915.08358268518</v>
+      </c>
+      <c r="N19" s="2">
+        <v>45915.08100641204</v>
+      </c>
+      <c r="O19" s="2">
+        <v>45915.18725445602</v>
+      </c>
+      <c r="P19" s="2">
+        <v>45915.26926759259</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>45915.37480168982</v>
+      </c>
+      <c r="R19" s="2">
+        <v>45915.60506037037</v>
+      </c>
+      <c r="T19" s="2">
+        <v>45915.97002079861</v>
+      </c>
+      <c r="V19" s="2">
+        <v>45916.20189703703</v>
+      </c>
+      <c r="W19" s="2">
+        <v>45916.39650483796</v>
+      </c>
+      <c r="X19" s="2">
+        <v>45916.45933371528</v>
+      </c>
+      <c r="Y19" s="2">
+        <v>45916.53816135417</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>45916.64014879629</v>
+      </c>
+      <c r="AA19" s="2">
+        <v>45916.78958375</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>45916.8618480787</v>
+      </c>
+      <c r="AC19" s="2">
+        <v>45916.96367357639</v>
+      </c>
+      <c r="AD19" s="2">
+        <v>45917.06572414352</v>
+      </c>
+      <c r="AE19" s="2">
+        <v>45917.23132472222</v>
+      </c>
+      <c r="AF19" s="2">
+        <v>45917.41728608796</v>
+      </c>
+      <c r="AG19" s="2">
+        <v>45917.5006153125</v>
+      </c>
+      <c r="AH19" s="2">
+        <v>45917.59454695602</v>
+      </c>
+      <c r="AI19" s="2">
+        <v>45917.71892535879</v>
+      </c>
+      <c r="AJ19" s="2">
+        <v>45917.82246778935</v>
+      </c>
+      <c r="AK19" s="2">
+        <v>45917.97690543981</v>
+      </c>
+      <c r="AL19" s="2">
+        <v>45918.10435318287</v>
+      </c>
+      <c r="AU19" s="2">
+        <v>45914.87498131944</v>
+      </c>
+      <c r="BF19" s="2">
+        <v>45920.46710648148</v>
+      </c>
+    </row>
+    <row r="20" spans="1:58">
+      <c r="A20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20">
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20">
+        <v>2023</v>
+      </c>
+      <c r="F20" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" t="s">
+        <v>89</v>
+      </c>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J20" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K20" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L20" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M20" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N20" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O20" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P20" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R20" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S20" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T20" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U20" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V20" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W20" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X20" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z20" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF20" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="21" spans="1:58">
+      <c r="A21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21">
+        <v>275</v>
+      </c>
+      <c r="C21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21">
+        <v>2023</v>
+      </c>
+      <c r="F21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G21" t="s">
+        <v>89</v>
+      </c>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J21" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K21" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L21" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M21" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N21" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O21" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P21" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R21" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S21" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T21" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U21" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V21" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W21" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X21" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y21" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z21" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA21" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB21" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC21" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD21" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE21" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF21" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG21" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK21" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF21" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="22" spans="1:58">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22">
+        <v>493</v>
+      </c>
+      <c r="C22" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22">
+        <v>2023</v>
+      </c>
+      <c r="F22" t="s">
+        <v>87</v>
+      </c>
+      <c r="G22" t="s">
+        <v>89</v>
+      </c>
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J22" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K22" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L22" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M22" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N22" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O22" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P22" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R22" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S22" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T22" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U22" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V22" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W22" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X22" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y22" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z22" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA22" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB22" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC22" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD22" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE22" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF22" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="23" spans="1:58">
+      <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23">
+        <v>540</v>
+      </c>
+      <c r="C23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23">
+        <v>2023</v>
+      </c>
+      <c r="F23" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J23" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K23" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L23" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M23" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N23" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O23" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF23" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="24" spans="1:58">
+      <c r="A24" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24">
+        <v>665</v>
+      </c>
+      <c r="C24" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24">
+        <v>2023</v>
+      </c>
+      <c r="F24" t="s">
+        <v>87</v>
+      </c>
+      <c r="G24" t="s">
+        <v>90</v>
+      </c>
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J24" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K24" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L24" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M24" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N24" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O24" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P24" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R24" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S24" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T24" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V24" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W24" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X24" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z24" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF24" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="25" spans="1:58">
+      <c r="A25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25">
+        <v>1105</v>
+      </c>
+      <c r="C25" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E25">
+        <v>2023</v>
+      </c>
+      <c r="F25" t="s">
+        <v>87</v>
+      </c>
+      <c r="G25" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J25" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K25" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L25" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M25" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N25" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O25" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R25" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S25" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF25" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="26" spans="1:58">
+      <c r="A26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26">
+        <v>1143</v>
+      </c>
+      <c r="C26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26">
+        <v>2023</v>
+      </c>
+      <c r="F26" t="s">
+        <v>87</v>
+      </c>
+      <c r="G26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J26" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K26" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L26" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M26" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N26" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O26" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R26" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S26" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T26" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U26" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V26" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W26" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X26" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y26" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z26" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA26" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB26" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD26" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE26" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF26" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG26" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF26" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="27" spans="1:58">
+      <c r="A27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27">
+        <v>1321</v>
+      </c>
+      <c r="C27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27">
+        <v>2023</v>
+      </c>
+      <c r="F27" t="s">
+        <v>87</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J27" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K27" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L27" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M27" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N27" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O27" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P27" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R27" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S27" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T27" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U27" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V27" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W27" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X27" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA27" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF27" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="28" spans="1:58">
+      <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28">
+        <v>48</v>
+      </c>
+      <c r="C28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28">
+        <v>2023</v>
+      </c>
+      <c r="F28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G28" t="s">
+        <v>89</v>
+      </c>
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J28" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K28" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L28" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M28" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N28" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O28" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P28" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R28" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S28" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T28" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U28" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V28" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W28" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X28" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z28" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF28" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="29" spans="1:58">
+      <c r="A29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29">
+        <v>275</v>
+      </c>
+      <c r="C29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29">
+        <v>2023</v>
+      </c>
+      <c r="F29" t="s">
+        <v>87</v>
+      </c>
+      <c r="G29" t="s">
+        <v>89</v>
+      </c>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J29" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K29" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L29" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M29" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N29" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O29" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P29" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R29" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S29" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T29" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U29" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V29" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W29" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X29" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y29" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z29" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA29" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB29" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC29" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD29" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE29" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF29" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG29" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK29" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF29" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="30" spans="1:58">
+      <c r="A30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30">
+        <v>493</v>
+      </c>
+      <c r="C30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30">
+        <v>2023</v>
+      </c>
+      <c r="F30" t="s">
+        <v>87</v>
+      </c>
+      <c r="G30" t="s">
+        <v>89</v>
+      </c>
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J30" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K30" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L30" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M30" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N30" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O30" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P30" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R30" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S30" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T30" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U30" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V30" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W30" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X30" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y30" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z30" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA30" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB30" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC30" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD30" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE30" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF30" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="31" spans="1:58">
+      <c r="A31" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31">
+        <v>540</v>
+      </c>
+      <c r="C31" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" t="s">
+        <v>79</v>
+      </c>
+      <c r="E31">
+        <v>2023</v>
+      </c>
+      <c r="F31" t="s">
+        <v>87</v>
+      </c>
+      <c r="G31" t="s">
+        <v>90</v>
+      </c>
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J31" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K31" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L31" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M31" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N31" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O31" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF31" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="32" spans="1:58">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32">
+        <v>665</v>
+      </c>
+      <c r="C32" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32">
+        <v>2023</v>
+      </c>
+      <c r="F32" t="s">
+        <v>87</v>
+      </c>
+      <c r="G32" t="s">
+        <v>90</v>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J32" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K32" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L32" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M32" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N32" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O32" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P32" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R32" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S32" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T32" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V32" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W32" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X32" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z32" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF32" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="33" spans="1:58">
+      <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33">
+        <v>1105</v>
+      </c>
+      <c r="C33" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" t="s">
+        <v>81</v>
+      </c>
+      <c r="E33">
+        <v>2023</v>
+      </c>
+      <c r="F33" t="s">
+        <v>87</v>
+      </c>
+      <c r="G33" t="s">
+        <v>90</v>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J33" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K33" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L33" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M33" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N33" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O33" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R33" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S33" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF33" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="34" spans="1:58">
+      <c r="A34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34">
+        <v>1143</v>
+      </c>
+      <c r="C34" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34">
+        <v>2023</v>
+      </c>
+      <c r="F34" t="s">
+        <v>87</v>
+      </c>
+      <c r="G34" t="s">
+        <v>91</v>
+      </c>
+      <c r="H34" t="b">
+        <v>1</v>
+      </c>
+      <c r="I34" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J34" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K34" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L34" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M34" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N34" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O34" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R34" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S34" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T34" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U34" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V34" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W34" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X34" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y34" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z34" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA34" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB34" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD34" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE34" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF34" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG34" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF34" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="35" spans="1:58">
+      <c r="A35" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35">
+        <v>1321</v>
+      </c>
+      <c r="C35" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35">
+        <v>2023</v>
+      </c>
+      <c r="F35" t="s">
+        <v>87</v>
+      </c>
+      <c r="G35" t="s">
+        <v>91</v>
+      </c>
+      <c r="H35" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J35" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K35" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L35" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M35" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N35" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O35" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P35" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R35" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S35" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T35" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U35" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V35" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W35" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X35" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA35" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF35" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="36" spans="1:58">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36">
+        <v>668</v>
+      </c>
+      <c r="C36" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36">
+        <v>2021</v>
+      </c>
+      <c r="F36" t="s">
+        <v>87</v>
+      </c>
+      <c r="G36" t="s">
+        <v>88</v>
+      </c>
+      <c r="H36" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2">
+        <v>44451.49266203704</v>
+      </c>
+      <c r="J36" s="2">
+        <v>44451.63459490741</v>
+      </c>
+      <c r="K36" s="2">
+        <v>44451.68247685185</v>
+      </c>
+      <c r="L36" s="2">
+        <v>44451.82474537037</v>
+      </c>
+      <c r="M36" s="2">
+        <v>44452.10481481482</v>
+      </c>
+      <c r="N36" s="2">
+        <v>44452.15012731482</v>
+      </c>
+      <c r="O36" s="2">
+        <v>44452.24664351852</v>
+      </c>
+      <c r="P36" s="2">
+        <v>44452.34168981481</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>44452.47001157407</v>
+      </c>
+      <c r="R36" s="2">
+        <v>44452.73408564815</v>
+      </c>
+      <c r="S36" s="2">
+        <v>44453.05474537037</v>
+      </c>
+      <c r="T36" s="2">
+        <v>44453.17554398148</v>
+      </c>
+      <c r="U36" s="2">
+        <v>44453.29359953704</v>
+      </c>
+      <c r="V36" s="2">
+        <v>44453.35523148148</v>
+      </c>
+      <c r="X36" s="2">
+        <v>44453.64238425926</v>
+      </c>
+      <c r="Y36" s="2">
+        <v>44453.73892361111</v>
+      </c>
+      <c r="Z36" s="2">
+        <v>44453.85755787037</v>
+      </c>
+      <c r="AA36" s="2">
+        <v>44453.9968287037</v>
+      </c>
+      <c r="AB36" s="2">
+        <v>44454.07862268519</v>
+      </c>
+      <c r="AC36" s="2">
+        <v>44454.20292824074</v>
+      </c>
+      <c r="AD36" s="2">
+        <v>44454.34174768518</v>
+      </c>
+      <c r="AE36" s="2">
+        <v>44454.54237268519</v>
+      </c>
+      <c r="AF36" s="2">
+        <v>44454.65358796297</v>
+      </c>
+      <c r="AG36" s="2">
+        <v>44454.779375</v>
+      </c>
+      <c r="AH36" s="2">
+        <v>44454.98438657408</v>
+      </c>
+      <c r="BF36" s="2">
+        <v>44457.64336805556</v>
+      </c>
+    </row>
+    <row r="37" spans="1:58">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>668</v>
+      </c>
+      <c r="C37" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" t="s">
+        <v>77</v>
+      </c>
+      <c r="E37">
+        <v>2021</v>
+      </c>
+      <c r="F37" t="s">
+        <v>87</v>
+      </c>
+      <c r="G37" t="s">
+        <v>88</v>
+      </c>
+      <c r="H37" t="b">
+        <v>1</v>
+      </c>
+      <c r="I37" s="2">
+        <v>44451.49266203704</v>
+      </c>
+      <c r="J37" s="2">
+        <v>44451.63459490741</v>
+      </c>
+      <c r="K37" s="2">
+        <v>44451.68247685185</v>
+      </c>
+      <c r="L37" s="2">
+        <v>44451.82474537037</v>
+      </c>
+      <c r="M37" s="2">
+        <v>44452.10481481482</v>
+      </c>
+      <c r="N37" s="2">
+        <v>44452.15012731482</v>
+      </c>
+      <c r="O37" s="2">
+        <v>44452.24664351852</v>
+      </c>
+      <c r="P37" s="2">
+        <v>44452.34168981481</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>44452.47001157407</v>
+      </c>
+      <c r="R37" s="2">
+        <v>44452.73408564815</v>
+      </c>
+      <c r="S37" s="2">
+        <v>44453.05474537037</v>
+      </c>
+      <c r="T37" s="2">
+        <v>44453.17554398148</v>
+      </c>
+      <c r="U37" s="2">
+        <v>44453.29359953704</v>
+      </c>
+      <c r="V37" s="2">
+        <v>44453.35523148148</v>
+      </c>
+      <c r="X37" s="2">
+        <v>44453.64238425926</v>
+      </c>
+      <c r="Y37" s="2">
+        <v>44453.73892361111</v>
+      </c>
+      <c r="Z37" s="2">
+        <v>44453.85755787037</v>
+      </c>
+      <c r="AA37" s="2">
+        <v>44453.9968287037</v>
+      </c>
+      <c r="AB37" s="2">
+        <v>44454.07862268519</v>
+      </c>
+      <c r="AC37" s="2">
+        <v>44454.20292824074</v>
+      </c>
+      <c r="AD37" s="2">
+        <v>44454.34174768518</v>
+      </c>
+      <c r="AE37" s="2">
+        <v>44454.54237268519</v>
+      </c>
+      <c r="AF37" s="2">
+        <v>44454.65358796297</v>
+      </c>
+      <c r="AG37" s="2">
+        <v>44454.779375</v>
+      </c>
+      <c r="AH37" s="2">
+        <v>44454.98438657408</v>
+      </c>
+      <c r="BF37" s="2">
+        <v>44457.64336805556</v>
+      </c>
+    </row>
+    <row r="38" spans="1:58">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>48</v>
+      </c>
+      <c r="C38" t="s">
+        <v>76</v>
+      </c>
+      <c r="D38" t="s">
+        <v>78</v>
+      </c>
+      <c r="E38">
+        <v>2023</v>
+      </c>
+      <c r="F38" t="s">
+        <v>87</v>
+      </c>
+      <c r="G38" t="s">
+        <v>89</v>
+      </c>
+      <c r="H38" t="b">
+        <v>1</v>
+      </c>
+      <c r="I38" s="2">
+        <v>45179.39792824074</v>
+      </c>
+      <c r="J38" s="2">
+        <v>45179.50267361111</v>
+      </c>
+      <c r="K38" s="2">
+        <v>45179.52646990741</v>
+      </c>
+      <c r="L38" s="2">
+        <v>45179.59795138889</v>
+      </c>
+      <c r="M38" s="2">
+        <v>45179.72765046296</v>
+      </c>
+      <c r="N38" s="2">
+        <v>45179.75509259259</v>
+      </c>
+      <c r="O38" s="2">
+        <v>45179.76221064815</v>
+      </c>
+      <c r="P38" s="2">
+        <v>45179.81621527778</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>45179.87998842593</v>
+      </c>
+      <c r="R38" s="2">
+        <v>45180.00331018519</v>
+      </c>
+      <c r="S38" s="2">
+        <v>45180.16604166666</v>
+      </c>
+      <c r="T38" s="2">
+        <v>45180.21908564815</v>
+      </c>
+      <c r="U38" s="2">
+        <v>45180.23003472222</v>
+      </c>
+      <c r="V38" s="2">
+        <v>45180.27650462963</v>
+      </c>
+      <c r="W38" s="2">
+        <v>45180.42538194444</v>
+      </c>
+      <c r="X38" s="2">
+        <v>45180.468125</v>
+      </c>
+      <c r="Z38" s="2">
+        <v>45180.58392361111</v>
+      </c>
+      <c r="BF38" s="2">
+        <v>45182.23497685185</v>
+      </c>
+    </row>
+    <row r="39" spans="1:58">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>275</v>
+      </c>
+      <c r="C39" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" t="s">
+        <v>79</v>
+      </c>
+      <c r="E39">
+        <v>2023</v>
+      </c>
+      <c r="F39" t="s">
+        <v>87</v>
+      </c>
+      <c r="G39" t="s">
+        <v>89</v>
+      </c>
+      <c r="H39" t="b">
+        <v>1</v>
+      </c>
+      <c r="I39" s="2">
+        <v>45179.38922453704</v>
+      </c>
+      <c r="J39" s="2">
+        <v>45179.54383101852</v>
+      </c>
+      <c r="K39" s="2">
+        <v>45179.58179398148</v>
+      </c>
+      <c r="L39" s="2">
+        <v>45179.70383101852</v>
+      </c>
+      <c r="M39" s="2">
+        <v>45179.94988425926</v>
+      </c>
+      <c r="N39" s="2">
+        <v>45179.99344907407</v>
+      </c>
+      <c r="O39" s="2">
+        <v>45179.9962037037</v>
+      </c>
+      <c r="P39" s="2">
+        <v>45180.10306712963</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>45180.2472337963</v>
+      </c>
+      <c r="R39" s="2">
+        <v>45180.53554398148</v>
+      </c>
+      <c r="S39" s="2">
+        <v>45180.90009259259</v>
+      </c>
+      <c r="T39" s="2">
+        <v>45181.00655092593</v>
+      </c>
+      <c r="U39" s="2">
+        <v>45181.20306712963</v>
+      </c>
+      <c r="V39" s="2">
+        <v>45181.27269675926</v>
+      </c>
+      <c r="W39" s="2">
+        <v>45181.55180555556</v>
+      </c>
+      <c r="X39" s="2">
+        <v>45181.63777777777</v>
+      </c>
+      <c r="Y39" s="2">
+        <v>45181.7540162037</v>
+      </c>
+      <c r="Z39" s="2">
+        <v>45181.89640046296</v>
+      </c>
+      <c r="AA39" s="2">
+        <v>45181.98230324074</v>
+      </c>
+      <c r="AB39" s="2">
+        <v>45182.08106481482</v>
+      </c>
+      <c r="AC39" s="2">
+        <v>45182.35355324074</v>
+      </c>
+      <c r="AD39" s="2">
+        <v>45182.45358796296</v>
+      </c>
+      <c r="AE39" s="2">
+        <v>45182.59913194444</v>
+      </c>
+      <c r="AF39" s="2">
+        <v>45182.72322916667</v>
+      </c>
+      <c r="AG39" s="2">
+        <v>45182.83815972223</v>
+      </c>
+      <c r="AK39" s="2">
+        <v>45183.06462962963</v>
+      </c>
+      <c r="BF39" s="2">
+        <v>45185.59189814814</v>
+      </c>
+    </row>
+    <row r="40" spans="1:58">
+      <c r="A40" t="s">
+        <v>61</v>
+      </c>
+      <c r="B40">
+        <v>493</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" t="s">
+        <v>77</v>
+      </c>
+      <c r="E40">
+        <v>2023</v>
+      </c>
+      <c r="F40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G40" t="s">
+        <v>89</v>
+      </c>
+      <c r="H40" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" s="2">
+        <v>45179.409375</v>
+      </c>
+      <c r="J40" s="2">
+        <v>45179.55034722222</v>
+      </c>
+      <c r="K40" s="2">
+        <v>45179.59763888889</v>
+      </c>
+      <c r="L40" s="2">
+        <v>45179.72980324074</v>
+      </c>
+      <c r="M40" s="2">
+        <v>45179.96844907408</v>
+      </c>
+      <c r="N40" s="2">
+        <v>45180.01599537037</v>
+      </c>
+      <c r="O40" s="2">
+        <v>45180.11148148148</v>
+      </c>
+      <c r="P40" s="2">
+        <v>45180.24331018519</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>45180.3828587963</v>
+      </c>
+      <c r="R40" s="2">
+        <v>45180.71607638889</v>
+      </c>
+      <c r="S40" s="2">
+        <v>45180.96011574074</v>
+      </c>
+      <c r="T40" s="2">
+        <v>45181.15980324074</v>
+      </c>
+      <c r="U40" s="2">
+        <v>45181.24869212963</v>
+      </c>
+      <c r="V40" s="2">
+        <v>45181.34960648148</v>
+      </c>
+      <c r="W40" s="2">
+        <v>45181.65403935185</v>
+      </c>
+      <c r="X40" s="2">
+        <v>45181.75313657407</v>
+      </c>
+      <c r="Y40" s="2">
+        <v>45181.81587962963</v>
+      </c>
+      <c r="Z40" s="2">
+        <v>45181.9002662037</v>
+      </c>
+      <c r="AA40" s="2">
+        <v>45181.90072916666</v>
+      </c>
+      <c r="AB40" s="2">
+        <v>45182.20228009259</v>
+      </c>
+      <c r="AC40" s="2">
+        <v>45182.37464120371</v>
+      </c>
+      <c r="AD40" s="2">
+        <v>45182.49806712963</v>
+      </c>
+      <c r="AE40" s="2">
+        <v>45182.64914351852</v>
+      </c>
+      <c r="BF40" s="2">
+        <v>45183.00606481481</v>
+      </c>
+    </row>
+    <row r="41" spans="1:58">
+      <c r="A41" t="s">
+        <v>62</v>
+      </c>
+      <c r="B41">
+        <v>540</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41">
+        <v>2023</v>
+      </c>
+      <c r="F41" t="s">
+        <v>87</v>
+      </c>
+      <c r="G41" t="s">
+        <v>90</v>
+      </c>
+      <c r="H41" t="b">
+        <v>1</v>
+      </c>
+      <c r="I41" s="2">
+        <v>45179.39790509259</v>
+      </c>
+      <c r="J41" s="2">
+        <v>45179.53548611111</v>
+      </c>
+      <c r="K41" s="2">
+        <v>45179.57420138889</v>
+      </c>
+      <c r="L41" s="2">
+        <v>45179.70348379629</v>
+      </c>
+      <c r="M41" s="2">
+        <v>45179.93878472222</v>
+      </c>
+      <c r="N41" s="2">
+        <v>45179.99392361111</v>
+      </c>
+      <c r="O41" s="2">
+        <v>45180.06231481482</v>
+      </c>
+      <c r="BF41" s="2">
+        <v>45182.84180555555</v>
+      </c>
+    </row>
+    <row r="42" spans="1:58">
+      <c r="A42" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42">
+        <v>665</v>
+      </c>
+      <c r="C42" t="s">
+        <v>76</v>
+      </c>
+      <c r="D42" t="s">
+        <v>80</v>
+      </c>
+      <c r="E42">
+        <v>2023</v>
+      </c>
+      <c r="F42" t="s">
+        <v>87</v>
+      </c>
+      <c r="G42" t="s">
+        <v>90</v>
+      </c>
+      <c r="H42" t="b">
+        <v>1</v>
+      </c>
+      <c r="I42" s="2">
+        <v>45179.39430555556</v>
+      </c>
+      <c r="J42" s="2">
+        <v>45179.50248842593</v>
+      </c>
+      <c r="K42" s="2">
+        <v>45179.528125</v>
+      </c>
+      <c r="L42" s="2">
+        <v>45179.60185185185</v>
+      </c>
+      <c r="M42" s="2">
+        <v>45179.73332175926</v>
+      </c>
+      <c r="N42" s="2">
+        <v>45179.76197916667</v>
+      </c>
+      <c r="O42" s="2">
+        <v>45179.7722337963</v>
+      </c>
+      <c r="P42" s="2">
+        <v>45179.82659722222</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>45179.88775462963</v>
+      </c>
+      <c r="R42" s="2">
+        <v>45180.0141087963</v>
+      </c>
+      <c r="S42" s="2">
+        <v>45180.17658564815</v>
+      </c>
+      <c r="T42" s="2">
+        <v>45180.2478125</v>
+      </c>
+      <c r="V42" s="2">
+        <v>45180.32322916666</v>
+      </c>
+      <c r="W42" s="2">
+        <v>45180.49724537037</v>
+      </c>
+      <c r="X42" s="2">
+        <v>45180.54726851852</v>
+      </c>
+      <c r="Z42" s="2">
+        <v>45180.58400462963</v>
+      </c>
+      <c r="BF42" s="2">
+        <v>45184.37396990741</v>
+      </c>
+    </row>
+    <row r="43" spans="1:58">
+      <c r="A43" t="s">
+        <v>64</v>
+      </c>
+      <c r="B43">
+        <v>1105</v>
+      </c>
+      <c r="C43" t="s">
+        <v>76</v>
+      </c>
+      <c r="D43" t="s">
+        <v>81</v>
+      </c>
+      <c r="E43">
+        <v>2023</v>
+      </c>
+      <c r="F43" t="s">
+        <v>87</v>
+      </c>
+      <c r="G43" t="s">
+        <v>90</v>
+      </c>
+      <c r="H43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I43" s="2">
+        <v>45179.49493055556</v>
+      </c>
+      <c r="J43" s="2">
+        <v>45179.64465277778</v>
+      </c>
+      <c r="K43" s="2">
+        <v>45179.68689814815</v>
+      </c>
+      <c r="L43" s="2">
+        <v>45179.81511574074</v>
+      </c>
+      <c r="M43" s="2">
+        <v>45180.12268518518</v>
+      </c>
+      <c r="N43" s="2">
+        <v>45180.19484953704</v>
+      </c>
+      <c r="O43" s="2">
+        <v>45180.25997685185</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>45180.52630787037</v>
+      </c>
+      <c r="R43" s="2">
+        <v>45180.82422453703</v>
+      </c>
+      <c r="S43" s="2">
+        <v>45181.24221064815</v>
+      </c>
+      <c r="BF43" s="2">
+        <v>45183.73302083334</v>
+      </c>
+    </row>
+    <row r="44" spans="1:58">
+      <c r="A44" t="s">
+        <v>65</v>
+      </c>
+      <c r="B44">
+        <v>1143</v>
+      </c>
+      <c r="C44" t="s">
+        <v>75</v>
+      </c>
+      <c r="D44" t="s">
+        <v>82</v>
+      </c>
+      <c r="E44">
+        <v>2023</v>
+      </c>
+      <c r="F44" t="s">
+        <v>87</v>
+      </c>
+      <c r="G44" t="s">
+        <v>91</v>
+      </c>
+      <c r="H44" t="b">
+        <v>1</v>
+      </c>
+      <c r="I44" s="2">
+        <v>45179.48607638889</v>
+      </c>
+      <c r="J44" s="2">
+        <v>45179.64658564814</v>
+      </c>
+      <c r="K44" s="2">
+        <v>45179.7028587963</v>
+      </c>
+      <c r="L44" s="2">
+        <v>45179.83604166667</v>
+      </c>
+      <c r="M44" s="2">
+        <v>45180.12891203703</v>
+      </c>
+      <c r="N44" s="2">
+        <v>45180.18069444445</v>
+      </c>
+      <c r="O44" s="2">
+        <v>45180.28619212963</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>45180.49460648148</v>
+      </c>
+      <c r="R44" s="2">
+        <v>45180.77678240741</v>
+      </c>
+      <c r="S44" s="2">
+        <v>45181.10384259259</v>
+      </c>
+      <c r="T44" s="2">
+        <v>45181.21434027778</v>
+      </c>
+      <c r="U44" s="2">
+        <v>45181.30199074074</v>
+      </c>
+      <c r="V44" s="2">
+        <v>45181.37020833333</v>
+      </c>
+      <c r="W44" s="2">
+        <v>45181.58256944444</v>
+      </c>
+      <c r="X44" s="2">
+        <v>45181.65321759259</v>
+      </c>
+      <c r="Y44" s="2">
+        <v>45181.74200231482</v>
+      </c>
+      <c r="Z44" s="2">
+        <v>45181.88</v>
+      </c>
+      <c r="AA44" s="2">
+        <v>45181.96909722222</v>
+      </c>
+      <c r="AB44" s="2">
+        <v>45182.0671412037</v>
+      </c>
+      <c r="AD44" s="2">
+        <v>45182.3734375</v>
+      </c>
+      <c r="AE44" s="2">
+        <v>45182.5744675926</v>
+      </c>
+      <c r="AF44" s="2">
+        <v>45182.66641203704</v>
+      </c>
+      <c r="AG44" s="2">
+        <v>45182.74886574074</v>
+      </c>
+      <c r="BF44" s="2">
+        <v>45185.71348379629</v>
+      </c>
+    </row>
+    <row r="45" spans="1:58">
+      <c r="A45" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45">
+        <v>1321</v>
+      </c>
+      <c r="C45" t="s">
+        <v>75</v>
+      </c>
+      <c r="D45" t="s">
+        <v>83</v>
+      </c>
+      <c r="E45">
+        <v>2023</v>
+      </c>
+      <c r="F45" t="s">
+        <v>87</v>
+      </c>
+      <c r="G45" t="s">
+        <v>91</v>
+      </c>
+      <c r="H45" t="b">
+        <v>1</v>
+      </c>
+      <c r="I45" s="2">
+        <v>45179.47435185185</v>
+      </c>
+      <c r="J45" s="2">
+        <v>45179.63296296296</v>
+      </c>
+      <c r="K45" s="2">
+        <v>45179.68140046296</v>
+      </c>
+      <c r="L45" s="2">
+        <v>45179.80612268519</v>
+      </c>
+      <c r="M45" s="2">
+        <v>45180.06925925926</v>
+      </c>
+      <c r="N45" s="2">
+        <v>45180.1246875</v>
+      </c>
+      <c r="O45" s="2">
+        <v>45180.17931712963</v>
+      </c>
+      <c r="P45" s="2">
+        <v>45180.28188657408</v>
+      </c>
+      <c r="Q45" s="2">
+        <v>45180.41796296297</v>
+      </c>
+      <c r="R45" s="2">
+        <v>45180.68553240741</v>
+      </c>
+      <c r="S45" s="2">
+        <v>45180.97909722223</v>
+      </c>
+      <c r="T45" s="2">
+        <v>45181.17892361111</v>
+      </c>
+      <c r="U45" s="2">
+        <v>45181.2145949074</v>
+      </c>
+      <c r="V45" s="2">
+        <v>45181.29107638889</v>
+      </c>
+      <c r="W45" s="2">
+        <v>45181.51983796297</v>
+      </c>
+      <c r="X45" s="2">
+        <v>45181.60017361111</v>
+      </c>
+      <c r="AA45" s="2">
+        <v>45181.72148148148</v>
+      </c>
+      <c r="BF45" s="2">
+        <v>45184.58322916667</v>
+      </c>
+    </row>
+    <row r="46" spans="1:58">
+      <c r="A46" t="s">
+        <v>67</v>
+      </c>
+      <c r="B46">
+        <v>99</v>
+      </c>
+      <c r="C46" t="s">
+        <v>75</v>
+      </c>
+      <c r="D46" t="s">
+        <v>84</v>
+      </c>
+      <c r="E46">
+        <v>2024</v>
+      </c>
+      <c r="F46" t="s">
+        <v>87</v>
+      </c>
+      <c r="G46" t="s">
+        <v>89</v>
+      </c>
+      <c r="H46" t="b">
+        <v>1</v>
+      </c>
+      <c r="I46" s="2">
+        <v>45543.4059375</v>
+      </c>
+      <c r="J46" s="2">
+        <v>45543.52394675926</v>
+      </c>
+      <c r="K46" s="2">
+        <v>45543.55820601852</v>
+      </c>
+      <c r="L46" s="2">
+        <v>45543.64599537037</v>
+      </c>
+      <c r="M46" s="2">
+        <v>45543.81885416667</v>
+      </c>
+      <c r="N46" s="2">
+        <v>45543.85825231481</v>
+      </c>
+      <c r="O46" s="2">
+        <v>45543.89254629629</v>
+      </c>
+      <c r="P46" s="2">
+        <v>45543.97118055556</v>
+      </c>
+      <c r="Q46" s="2">
+        <v>45544.0574537037</v>
+      </c>
+      <c r="R46" s="2">
+        <v>45544.2559837963</v>
+      </c>
+      <c r="S46" s="2">
+        <v>45544.48283564814</v>
+      </c>
+      <c r="T46" s="2">
+        <v>45544.54177083333</v>
+      </c>
+      <c r="V46" s="2">
+        <v>45544.65012731482</v>
+      </c>
+      <c r="X46" s="2">
+        <v>45544.84173611111</v>
+      </c>
+      <c r="Y46" s="2">
+        <v>45544.90390046296</v>
+      </c>
+      <c r="Z46" s="2">
+        <v>45544.99487268519</v>
+      </c>
+      <c r="AA46" s="2">
+        <v>45545.21025462963</v>
+      </c>
+      <c r="AB46" s="2">
+        <v>45545.27203703704</v>
+      </c>
+      <c r="AC46" s="2">
+        <v>45545.35291666666</v>
+      </c>
+      <c r="AD46" s="2">
+        <v>45545.42675925926</v>
+      </c>
+      <c r="AE46" s="2">
+        <v>45545.54788194445</v>
+      </c>
+      <c r="AF46" s="2">
+        <v>45545.63417824074</v>
+      </c>
+      <c r="AG46" s="2">
+        <v>45545.70618055556</v>
+      </c>
+      <c r="AH46" s="2">
+        <v>45545.795</v>
+      </c>
+      <c r="AI46" s="2">
+        <v>45545.89577546297</v>
+      </c>
+      <c r="AJ46" s="2">
+        <v>45545.96357638889</v>
+      </c>
+      <c r="AK46" s="2">
+        <v>45546.15805555556</v>
+      </c>
+      <c r="AL46" s="2">
+        <v>45546.21180555555</v>
+      </c>
+      <c r="AM46" s="2">
+        <v>45546.41456018519</v>
+      </c>
+      <c r="BF46" s="2">
+        <v>45549.13998842592</v>
+      </c>
+    </row>
+    <row r="47" spans="1:58">
+      <c r="A47" t="s">
+        <v>68</v>
+      </c>
+      <c r="B47">
+        <v>1547</v>
+      </c>
+      <c r="C47" t="s">
+        <v>75</v>
+      </c>
+      <c r="D47" t="s">
+        <v>85</v>
+      </c>
+      <c r="E47">
+        <v>2024</v>
+      </c>
+      <c r="F47" t="s">
+        <v>87</v>
+      </c>
+      <c r="G47" t="s">
+        <v>89</v>
+      </c>
+      <c r="H47" t="b">
+        <v>1</v>
+      </c>
+      <c r="I47" s="2">
+        <v>45543.49523148148</v>
+      </c>
+      <c r="J47" s="2">
+        <v>45543.61390046297</v>
+      </c>
+      <c r="K47" s="2">
+        <v>45543.64502314815</v>
+      </c>
+      <c r="L47" s="2">
+        <v>45543.74020833334</v>
+      </c>
+      <c r="M47" s="2">
+        <v>45543.94842592593</v>
+      </c>
+      <c r="N47" s="2">
+        <v>45544.00671296296</v>
+      </c>
+      <c r="O47" s="2">
+        <v>45544.03377314815</v>
+      </c>
+      <c r="P47" s="2">
+        <v>45544.12354166667</v>
+      </c>
+      <c r="Q47" s="2">
+        <v>45544.24116898148</v>
+      </c>
+      <c r="R47" s="2">
+        <v>45544.51748842592</v>
+      </c>
+      <c r="S47" s="2">
+        <v>45544.86471064815</v>
+      </c>
+      <c r="T47" s="2">
+        <v>45545.03194444445</v>
+      </c>
+      <c r="U47" s="2">
+        <v>45545.28653935185</v>
+      </c>
+      <c r="BF47" s="2">
+        <v>45548.75009259259</v>
+      </c>
+    </row>
+    <row r="48" spans="1:58">
+      <c r="A48" t="s">
+        <v>71</v>
+      </c>
+      <c r="B48" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48" t="s">
+        <v>85</v>
+      </c>
+      <c r="E48" t="s">
+        <v>86</v>
+      </c>
+      <c r="F48" t="s">
+        <v>87</v>
+      </c>
+      <c r="G48" t="s">
+        <v>88</v>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" s="2">
+        <v>45914.47542606481</v>
+      </c>
+      <c r="J48" s="2">
+        <v>45914.62513768519</v>
+      </c>
+      <c r="K48" s="2">
+        <v>45914.66811888889</v>
+      </c>
+      <c r="L48" s="2">
+        <v>45914.7943594676</v>
+      </c>
+      <c r="M48" s="2">
+        <v>45915.11259197917</v>
+      </c>
+      <c r="N48" s="2">
+        <v>45915.18046519676</v>
+      </c>
+      <c r="O48" s="2">
+        <v>45915.23756817129</v>
+      </c>
+      <c r="P48" s="2">
+        <v>45915.33654960648</v>
+      </c>
+      <c r="Q48" s="2">
+        <v>45915.46181254629</v>
+      </c>
+      <c r="R48" s="2">
+        <v>45915.75465270833</v>
+      </c>
+      <c r="T48" s="2">
+        <v>45916.23184403935</v>
+      </c>
+      <c r="U48" s="2">
+        <v>45916.2964321875</v>
+      </c>
+      <c r="V48" s="2">
+        <v>45916.3633465625</v>
+      </c>
+      <c r="W48" s="2">
+        <v>45916.59064263889</v>
+      </c>
+      <c r="X48" s="2">
+        <v>45916.67155491898</v>
+      </c>
+      <c r="Y48" s="2">
+        <v>45916.76256023148</v>
+      </c>
+      <c r="Z48" s="2">
+        <v>45916.87893012731</v>
+      </c>
+      <c r="AA48" s="2">
+        <v>45917.01325516203</v>
+      </c>
+      <c r="AB48" s="2">
+        <v>45917.09894671296</v>
+      </c>
+      <c r="AC48" s="2">
+        <v>45917.2452054051</v>
+      </c>
+      <c r="AD48" s="2">
+        <v>45917.37764478009</v>
+      </c>
+      <c r="AE48" s="2">
+        <v>45917.56345918981</v>
+      </c>
+      <c r="AG48" s="2">
+        <v>45917.86822302084</v>
+      </c>
+      <c r="AU48" s="2">
+        <v>45914.91300321759</v>
+      </c>
+      <c r="BF48" s="2">
+        <v>45920.66509259259</v>
+      </c>
+    </row>
+    <row r="49" spans="1:58">
+      <c r="A49" t="s">
+        <v>72</v>
+      </c>
+      <c r="B49" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" t="s">
+        <v>76</v>
+      </c>
+      <c r="D49" t="s">
+        <v>82</v>
+      </c>
+      <c r="E49" t="s">
+        <v>86</v>
+      </c>
+      <c r="F49" t="s">
+        <v>87</v>
+      </c>
+      <c r="G49" t="s">
+        <v>89</v>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" s="2">
+        <v>45914.48986140046</v>
+      </c>
+      <c r="J49" s="2">
+        <v>45914.63592015046</v>
+      </c>
+      <c r="K49" s="2">
+        <v>45914.67685524306</v>
+      </c>
+      <c r="L49" s="2">
+        <v>45914.78852579861</v>
+      </c>
+      <c r="M49" s="2">
+        <v>45915.08358268518</v>
+      </c>
+      <c r="N49" s="2">
+        <v>45915.08100641204</v>
+      </c>
+      <c r="O49" s="2">
+        <v>45915.18725445602</v>
+      </c>
+      <c r="P49" s="2">
+        <v>45915.26926759259</v>
+      </c>
+      <c r="Q49" s="2">
+        <v>45915.37480168982</v>
+      </c>
+      <c r="R49" s="2">
+        <v>45915.60506037037</v>
+      </c>
+      <c r="T49" s="2">
+        <v>45915.97002079861</v>
+      </c>
+      <c r="V49" s="2">
+        <v>45916.20189703703</v>
+      </c>
+      <c r="W49" s="2">
+        <v>45916.39650483796</v>
+      </c>
+      <c r="X49" s="2">
+        <v>45916.45933371528</v>
+      </c>
+      <c r="Y49" s="2">
+        <v>45916.53816135417</v>
+      </c>
+      <c r="Z49" s="2">
+        <v>45916.64014879629</v>
+      </c>
+      <c r="AA49" s="2">
+        <v>45916.78958375</v>
+      </c>
+      <c r="AB49" s="2">
+        <v>45916.8618480787</v>
+      </c>
+      <c r="AC49" s="2">
+        <v>45916.96367357639</v>
+      </c>
+      <c r="AD49" s="2">
+        <v>45917.06572414352</v>
+      </c>
+      <c r="AE49" s="2">
+        <v>45917.23132472222</v>
+      </c>
+      <c r="AF49" s="2">
+        <v>45917.41728608796</v>
+      </c>
+      <c r="AG49" s="2">
+        <v>45917.5006153125</v>
+      </c>
+      <c r="AH49" s="2">
+        <v>45917.59454695602</v>
+      </c>
+      <c r="AI49" s="2">
+        <v>45917.71892535879</v>
+      </c>
+      <c r="AJ49" s="2">
+        <v>45917.82246778935</v>
+      </c>
+      <c r="AK49" s="2">
+        <v>45917.97690543981</v>
+      </c>
+      <c r="AL49" s="2">
+        <v>45918.10435318287</v>
+      </c>
+      <c r="AU49" s="2">
+        <v>45914.87498131944</v>
+      </c>
+      <c r="BF49" s="2">
+        <v>45920.46710648148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>